<commit_message>
Afegit any venda en "pigDeLaCompraEsElBooooo". Una compra pot tenir vendes en diferents anys.
</commit_message>
<xml_diff>
--- a/Docs/Proves-PiG Origen.xlsx
+++ b/Docs/Proves-PiG Origen.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\Meus\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76F15BB-757C-4BCE-940B-AD79AB20B64D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E43DB364-106D-4065-9D3D-D7129F382482}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{A356EC3C-A36B-4D01-97F4-538073D64CD4}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{A356EC3C-A36B-4D01-97F4-538073D64CD4}"/>
   </bookViews>
   <sheets>
-    <sheet name="Arcelor" sheetId="6" r:id="rId1"/>
-    <sheet name="Aberdeen Standard" sheetId="7" r:id="rId2"/>
-    <sheet name="27-Global Technology" sheetId="2" r:id="rId3"/>
-    <sheet name="29-CS Corto Plazo" sheetId="3" r:id="rId4"/>
-    <sheet name="Comparacio Aplic-Web" sheetId="5" r:id="rId5"/>
+    <sheet name="Proves" sheetId="8" r:id="rId1"/>
+    <sheet name="Arcelor" sheetId="6" r:id="rId2"/>
+    <sheet name="Aberdeen Standard" sheetId="7" r:id="rId3"/>
+    <sheet name="27-Global Technology" sheetId="2" r:id="rId4"/>
+    <sheet name="29-CS Corto Plazo" sheetId="3" r:id="rId5"/>
+    <sheet name="Comparacio Aplic-Web" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="50">
   <si>
     <t>Id</t>
   </si>
@@ -150,13 +151,50 @@
   </si>
   <si>
     <t>PiG Brut</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En cartera </t>
+  </si>
+  <si>
+    <t>PiG vendes reals</t>
+  </si>
+  <si>
+    <t>Pig Vendes reals + en cartera</t>
+  </si>
+  <si>
+    <t>Pig Nomes en cartera</t>
+  </si>
+  <si>
+    <t>v real</t>
+  </si>
+  <si>
+    <t>nomesPartsEnCartera</t>
+  </si>
+  <si>
+    <t>pigOrigen</t>
+  </si>
+  <si>
+    <t>NULL</t>
+  </si>
+  <si>
+    <t>v</t>
+  </si>
+  <si>
+    <t>c1-&gt;5</t>
+  </si>
+  <si>
+    <t>c1-&gt;5; c2-&gt;10; c3-&gt;5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="6">
+    <numFmt numFmtId="6" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="164" formatCode="#,##0.000\ &quot;€&quot;"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
@@ -315,7 +353,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -380,6 +418,8 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -693,19 +733,229 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35931D83-0E0A-4D88-B489-4583A6E933E1}">
-  <dimension ref="A1:Q25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D44DFC7A-A8B1-46AB-BBD2-1EFF59E4C2EB}">
+  <dimension ref="A1:J17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="1.90625" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.54296875" customWidth="1"/>
+    <col min="16" max="17" width="11.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2">
+        <v>100</v>
+      </c>
+      <c r="E2" s="40">
+        <v>11</v>
+      </c>
+      <c r="F2" s="40">
+        <f>D2*E2</f>
+        <v>1100</v>
+      </c>
+      <c r="G2" s="40"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3">
+        <v>80</v>
+      </c>
+      <c r="E3" s="40">
+        <v>9</v>
+      </c>
+      <c r="F3" s="40">
+        <f>D3*E2</f>
+        <v>880</v>
+      </c>
+      <c r="G3" s="40">
+        <f>D3*E3</f>
+        <v>720</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4">
+        <v>20</v>
+      </c>
+      <c r="E4" s="40">
+        <v>13</v>
+      </c>
+      <c r="F4" s="40">
+        <f>+D4*E2</f>
+        <v>220</v>
+      </c>
+      <c r="G4" s="40">
+        <f>D4*E4</f>
+        <v>260</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="I5" s="40" t="s">
+        <v>44</v>
+      </c>
+      <c r="J5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="40">
+        <f>D3*E3-D3*E2</f>
+        <v>-160</v>
+      </c>
+      <c r="F6" s="40">
+        <f>G3-F3</f>
+        <v>-160</v>
+      </c>
+      <c r="G6" s="40"/>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="40">
+        <f>D4*E4-D4*E2</f>
+        <v>40</v>
+      </c>
+      <c r="F7" s="40">
+        <f>G4-F4</f>
+        <v>40</v>
+      </c>
+      <c r="G7" s="40"/>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="40">
+        <f>E6+D4*E4-D4*E2</f>
+        <v>-120</v>
+      </c>
+      <c r="F8" s="40">
+        <f>SUM(F6:F7)</f>
+        <v>-120</v>
+      </c>
+      <c r="G8" s="40"/>
+      <c r="I8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>1</v>
+      </c>
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>2</v>
+      </c>
+      <c r="B14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>3</v>
+      </c>
+      <c r="B15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16">
+        <v>5</v>
+      </c>
+      <c r="E16" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17">
+        <v>20</v>
+      </c>
+      <c r="E17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35931D83-0E0A-4D88-B489-4583A6E933E1}">
+  <dimension ref="A1:Q34"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.1796875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="1.90625" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="7" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="10.54296875" customWidth="1"/>
     <col min="16" max="17" width="11.1796875" bestFit="1" customWidth="1"/>
   </cols>
@@ -765,6 +1015,10 @@
         <f>D2</f>
         <v>925</v>
       </c>
+      <c r="L2" s="5">
+        <f>+G3-G2</f>
+        <v>167.73999999999978</v>
+      </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A3" s="30">
@@ -1375,6 +1629,7 @@
         <f t="shared" si="0"/>
         <v>992</v>
       </c>
+      <c r="K19" s="34"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="30">
@@ -1408,6 +1663,10 @@
         <f t="shared" si="0"/>
         <v>1652</v>
       </c>
+      <c r="K20" s="34">
+        <v>400</v>
+      </c>
+      <c r="L20" s="34"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="30">
@@ -1441,6 +1700,8 @@
         <f>J20-D21</f>
         <v>400</v>
       </c>
+      <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="30">
@@ -1474,6 +1735,13 @@
         <f t="shared" si="0"/>
         <v>967</v>
       </c>
+      <c r="K22" s="34">
+        <f>D22</f>
+        <v>567</v>
+      </c>
+      <c r="L22" s="34">
+        <v>67</v>
+      </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="30">
@@ -1507,6 +1775,14 @@
         <f t="shared" si="0"/>
         <v>1467</v>
       </c>
+      <c r="K23" s="34">
+        <f>D23</f>
+        <v>500</v>
+      </c>
+      <c r="L23" s="34">
+        <f t="shared" ref="L23:L25" si="1">K23</f>
+        <v>500</v>
+      </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="30">
@@ -1540,6 +1816,14 @@
         <f t="shared" si="0"/>
         <v>1900</v>
       </c>
+      <c r="K24" s="34">
+        <f>D24</f>
+        <v>433</v>
+      </c>
+      <c r="L24" s="34">
+        <f t="shared" si="1"/>
+        <v>433</v>
+      </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="30">
@@ -1572,6 +1856,168 @@
       <c r="J25" s="34">
         <f t="shared" si="0"/>
         <v>1900</v>
+      </c>
+      <c r="K25" s="34">
+        <f>D25</f>
+        <v>0</v>
+      </c>
+      <c r="L25" s="34">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="K26" s="41">
+        <f>SUM(K20:K25)</f>
+        <v>1900</v>
+      </c>
+      <c r="L26" s="41">
+        <f>SUM(L20:L25)</f>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="E29" s="40"/>
+      <c r="F29" s="40"/>
+      <c r="G29" s="40"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="E30" s="40"/>
+      <c r="F30" s="40"/>
+      <c r="G30" s="40"/>
+      <c r="J30" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A31" s="30">
+        <v>166</v>
+      </c>
+      <c r="B31" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="C31" s="31">
+        <v>43389</v>
+      </c>
+      <c r="D31" s="33">
+        <v>1600</v>
+      </c>
+      <c r="E31" s="32">
+        <v>24.388000000000002</v>
+      </c>
+      <c r="F31" s="32">
+        <v>39020.800000000003</v>
+      </c>
+      <c r="G31" s="32">
+        <v>39049.31</v>
+      </c>
+      <c r="H31" s="30">
+        <v>1</v>
+      </c>
+      <c r="I31" s="32">
+        <v>28.51</v>
+      </c>
+      <c r="J31" s="34"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A32" s="30">
+        <v>169</v>
+      </c>
+      <c r="B32" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" s="31">
+        <v>43458</v>
+      </c>
+      <c r="D32" s="33">
+        <v>648</v>
+      </c>
+      <c r="E32" s="32">
+        <v>18.260000000000002</v>
+      </c>
+      <c r="F32" s="32">
+        <v>11832.48</v>
+      </c>
+      <c r="G32" s="32">
+        <v>11822.42</v>
+      </c>
+      <c r="H32" s="30">
+        <v>1</v>
+      </c>
+      <c r="I32" s="32">
+        <v>10.06</v>
+      </c>
+      <c r="J32" s="32">
+        <f>G$31/D$31*D32</f>
+        <v>15814.970549999998</v>
+      </c>
+      <c r="L32" s="5">
+        <f>+G32-J32</f>
+        <v>-3992.5505499999981</v>
+      </c>
+      <c r="M32" s="5">
+        <v>-3992.5505499999899</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A33" s="30">
+        <v>177</v>
+      </c>
+      <c r="B33" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33" s="31">
+        <v>43797</v>
+      </c>
+      <c r="D33" s="33">
+        <f>+D31-D32</f>
+        <v>952</v>
+      </c>
+      <c r="E33" s="32">
+        <v>15.624000000000001</v>
+      </c>
+      <c r="F33" s="32">
+        <f>D33*E33</f>
+        <v>14874.048000000001</v>
+      </c>
+      <c r="G33" s="32">
+        <f>F33-I33</f>
+        <v>14866.39854313099</v>
+      </c>
+      <c r="H33" s="30">
+        <v>1</v>
+      </c>
+      <c r="I33" s="32">
+        <f>10.06/D17*D33</f>
+        <v>7.6494568690095841</v>
+      </c>
+      <c r="J33" s="32">
+        <f>G$31/D$31*D33</f>
+        <v>23234.339449999999</v>
+      </c>
+      <c r="L33" s="5">
+        <f>+G33-J33</f>
+        <v>-8367.9409068690093</v>
+      </c>
+      <c r="M33" s="5">
+        <v>-8367.9409068690093</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="G34" s="5"/>
+      <c r="L34" s="29">
+        <f>SUM(L32:L33)</f>
+        <v>-12360.491456869007</v>
+      </c>
+      <c r="M34" s="29">
+        <f>SUM(M32:M33)</f>
+        <v>-12360.491456869</v>
       </c>
     </row>
   </sheetData>
@@ -1580,7 +2026,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2765C9F5-04DD-4DF6-B6C4-239116C295E5}">
   <dimension ref="A1:I100"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1863,7 +2309,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8A68C22-9B46-4722-8C3E-CFEEA15AC7BA}">
   <dimension ref="A1:J42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2646,7 +3092,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2C274DA-F909-48E4-B094-8A2D400FEEEF}">
   <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2848,7 +3294,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B93F3808-9942-41FF-8964-468989940CAA}">
   <dimension ref="B1:J28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Calcula PiG en cartera
--HG--
branch : Nou Càlcul pigVendesReals
</commit_message>
<xml_diff>
--- a/Docs/Proves-PiG Origen.xlsx
+++ b/Docs/Proves-PiG Origen.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\Meus\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F9E0640-EEA2-4DF8-9153-637D67AB0898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF39A4F-8DD9-4A1A-B8C2-E5C22E9D0CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{A356EC3C-A36B-4D01-97F4-538073D64CD4}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{A356EC3C-A36B-4D01-97F4-538073D64CD4}"/>
   </bookViews>
   <sheets>
-    <sheet name="PiG 2015" sheetId="9" r:id="rId1"/>
-    <sheet name="Proves" sheetId="8" r:id="rId2"/>
-    <sheet name="Arcelor" sheetId="6" r:id="rId3"/>
-    <sheet name="Aberdeen Standard" sheetId="7" r:id="rId4"/>
-    <sheet name="27-Global Technology" sheetId="2" r:id="rId5"/>
-    <sheet name="29-CS Corto Plazo" sheetId="3" r:id="rId6"/>
-    <sheet name="Comparacio Aplic-Web" sheetId="5" r:id="rId7"/>
+    <sheet name="Asian Smaller" sheetId="10" r:id="rId1"/>
+    <sheet name="PiG 2015" sheetId="9" r:id="rId2"/>
+    <sheet name="Proves" sheetId="8" r:id="rId3"/>
+    <sheet name="Arcelor" sheetId="6" r:id="rId4"/>
+    <sheet name="Aberdeen Standard" sheetId="7" r:id="rId5"/>
+    <sheet name="27-Global Technology" sheetId="2" r:id="rId6"/>
+    <sheet name="29-CS Corto Plazo" sheetId="3" r:id="rId7"/>
+    <sheet name="Comparacio Aplic-Web" sheetId="5" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="77">
   <si>
     <t>Id</t>
   </si>
@@ -133,9 +134,6 @@
     <t>Dif totsl</t>
   </si>
   <si>
-    <t>ContraSplit</t>
-  </si>
-  <si>
     <t>Dividends</t>
   </si>
   <si>
@@ -212,19 +210,82 @@
   </si>
   <si>
     <t>Dif PiG</t>
+  </si>
+  <si>
+    <t>Vendes Net</t>
+  </si>
+  <si>
+    <t>Compres Net</t>
+  </si>
+  <si>
+    <t>V4</t>
+  </si>
+  <si>
+    <t>V5</t>
+  </si>
+  <si>
+    <t>V6</t>
+  </si>
+  <si>
+    <t>V95</t>
+  </si>
+  <si>
+    <t>V187</t>
+  </si>
+  <si>
+    <t>6-Biotechnology C USD Acc</t>
+  </si>
+  <si>
+    <t>Asian Smaller</t>
+  </si>
+  <si>
+    <t>PiG Orig</t>
+  </si>
+  <si>
+    <t>PU Orig</t>
+  </si>
+  <si>
+    <t>Cost Orig</t>
+  </si>
+  <si>
+    <t>Fons</t>
+  </si>
+  <si>
+    <t>Accions</t>
+  </si>
+  <si>
+    <t>En Cartera</t>
+  </si>
+  <si>
+    <t>A SelfBank</t>
+  </si>
+  <si>
+    <t>En l'app</t>
+  </si>
+  <si>
+    <t>ContSplit</t>
+  </si>
+  <si>
+    <t>PiG Apl</t>
+  </si>
+  <si>
+    <t>PiG no desp</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="9">
     <numFmt numFmtId="6" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="164" formatCode="#,##0.000\ &quot;€&quot;"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="#,##0.000"/>
     <numFmt numFmtId="167" formatCode="#,##0.0000\ _€"/>
+    <numFmt numFmtId="168" formatCode="#,##0.000\ &quot;€&quot;;[Red]\-#,##0.000\ &quot;€&quot;"/>
+    <numFmt numFmtId="169" formatCode="#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="170" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -243,7 +304,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -277,6 +338,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -390,7 +457,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -458,14 +525,29 @@
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="8" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="8" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="170" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="170" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -779,6 +861,614 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0833B7FE-9444-4F79-99B0-FA4EF66F88D9}">
+  <dimension ref="A1:R22"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="3.90625" style="48" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.6328125" customWidth="1"/>
+    <col min="8" max="8" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="1.54296875" customWidth="1"/>
+    <col min="10" max="11" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="1.90625" customWidth="1"/>
+    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A1" s="2"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A2" s="49" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="Q2" s="2"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A3" s="47">
+        <v>1</v>
+      </c>
+      <c r="B3" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="31">
+        <v>41172</v>
+      </c>
+      <c r="D3" s="45">
+        <v>325.52199999999999</v>
+      </c>
+      <c r="E3" s="32">
+        <v>30.719899999999999</v>
+      </c>
+      <c r="F3" s="32">
+        <v>9999.99</v>
+      </c>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="J3" s="15">
+        <f>D3</f>
+        <v>325.52199999999999</v>
+      </c>
+      <c r="K3" s="15">
+        <f>D3</f>
+        <v>325.52199999999999</v>
+      </c>
+      <c r="Q3" s="46">
+        <f>K3*E6-F3</f>
+        <v>1062.3543348000003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A4" s="47">
+        <v>2</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="31">
+        <v>41187</v>
+      </c>
+      <c r="D4" s="45">
+        <v>1267.6880000000001</v>
+      </c>
+      <c r="E4" s="32">
+        <v>31.5535</v>
+      </c>
+      <c r="F4" s="32">
+        <v>39999.980000000003</v>
+      </c>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="J4" s="15">
+        <f>J3+D4</f>
+        <v>1593.21</v>
+      </c>
+      <c r="K4" s="15">
+        <f>D6-K3</f>
+        <v>1090.0600000000002</v>
+      </c>
+      <c r="L4" s="15">
+        <f>D4-K4</f>
+        <v>177.62799999999993</v>
+      </c>
+      <c r="M4" s="15"/>
+      <c r="Q4" s="46">
+        <f>K4*E6+L4*E7-F4</f>
+        <v>3064.9147432000027</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A5" s="47">
+        <v>3</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="31">
+        <v>41410</v>
+      </c>
+      <c r="D5" s="45">
+        <v>522.37400000000002</v>
+      </c>
+      <c r="E5" s="32">
+        <v>38.286799999999999</v>
+      </c>
+      <c r="F5" s="32">
+        <v>20000.02</v>
+      </c>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="J5" s="15">
+        <f>J4+D5</f>
+        <v>2115.5839999999998</v>
+      </c>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15">
+        <f>D7-L4</f>
+        <v>0.37200000000007094</v>
+      </c>
+      <c r="M5" s="15">
+        <f>D5-L5</f>
+        <v>522.00199999999995</v>
+      </c>
+      <c r="Q5" s="46">
+        <f>L5*E7+M5*E8-F5</f>
+        <v>-3037.8489985999986</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A6" s="47">
+        <v>4</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="31">
+        <v>41438</v>
+      </c>
+      <c r="D6" s="45">
+        <v>1415.5820000000001</v>
+      </c>
+      <c r="E6" s="32">
+        <v>33.983400000000003</v>
+      </c>
+      <c r="F6" s="32">
+        <v>48106.28</v>
+      </c>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="J6" s="15">
+        <f>J5-D6</f>
+        <v>700.00199999999973</v>
+      </c>
+      <c r="L6" s="15"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A7" s="47">
+        <v>5</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="31">
+        <v>41492</v>
+      </c>
+      <c r="D7" s="45">
+        <v>178</v>
+      </c>
+      <c r="E7" s="32">
+        <v>33.8964</v>
+      </c>
+      <c r="F7" s="32">
+        <v>6033.56</v>
+      </c>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="J7" s="15">
+        <f>J6-D7</f>
+        <v>522.00199999999973</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A8" s="47">
+        <v>6</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="31">
+        <v>41506</v>
+      </c>
+      <c r="D8" s="45">
+        <v>522.00199999999995</v>
+      </c>
+      <c r="E8" s="32">
+        <v>32.470300000000002</v>
+      </c>
+      <c r="F8" s="32">
+        <v>16949.560000000001</v>
+      </c>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="J8" s="15">
+        <f>J7-D8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A9" s="47">
+        <v>41</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="31">
+        <v>42047</v>
+      </c>
+      <c r="D9" s="45">
+        <v>174.22900000000001</v>
+      </c>
+      <c r="E9" s="32">
+        <v>39.429099999999998</v>
+      </c>
+      <c r="F9" s="32">
+        <v>6869.7</v>
+      </c>
+      <c r="G9" s="32">
+        <f>D16</f>
+        <v>15</v>
+      </c>
+      <c r="H9" s="32">
+        <f>E16</f>
+        <v>457.97989999999999</v>
+      </c>
+      <c r="J9" s="15">
+        <f>J8+D9</f>
+        <v>174.22900000000001</v>
+      </c>
+      <c r="N9" s="15">
+        <f>D10</f>
+        <v>150</v>
+      </c>
+      <c r="O9" s="15">
+        <f>D9-D10</f>
+        <v>24.229000000000013</v>
+      </c>
+      <c r="P9" s="15"/>
+      <c r="Q9" s="46">
+        <f>F11-O9*E9</f>
+        <v>74.792336099999375</v>
+      </c>
+      <c r="R9" s="46">
+        <f>F11-Q16</f>
+        <v>507.70927892601082</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A10" s="47">
+        <v>95</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="31">
+        <v>42207</v>
+      </c>
+      <c r="D10" s="45">
+        <v>150</v>
+      </c>
+      <c r="E10" s="32">
+        <v>39.5777</v>
+      </c>
+      <c r="F10" s="32">
+        <v>5936.65</v>
+      </c>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="J10" s="15">
+        <f>J9-D10</f>
+        <v>24.229000000000013</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A11" s="47">
+        <v>187</v>
+      </c>
+      <c r="B11" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="31">
+        <v>44176</v>
+      </c>
+      <c r="D11" s="45">
+        <v>24.228999999999999</v>
+      </c>
+      <c r="E11" s="32">
+        <v>42.515799999999999</v>
+      </c>
+      <c r="F11" s="32">
+        <v>1030.1199999999999</v>
+      </c>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="J11" s="15">
+        <f>J10-D11</f>
+        <v>0</v>
+      </c>
+      <c r="R11" s="46"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="R12" s="5"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A13" s="49" t="s">
+        <v>64</v>
+      </c>
+      <c r="R13" s="5"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A14" s="30">
+        <v>7</v>
+      </c>
+      <c r="B14" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="31">
+        <v>41492</v>
+      </c>
+      <c r="D14" s="30">
+        <v>24.091999999999999</v>
+      </c>
+      <c r="E14" s="32">
+        <v>250.44120000000001</v>
+      </c>
+      <c r="F14" s="32">
+        <v>6033.63</v>
+      </c>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="J14" s="15">
+        <f>D14</f>
+        <v>24.091999999999999</v>
+      </c>
+      <c r="K14" s="15"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A15" s="30">
+        <v>39</v>
+      </c>
+      <c r="B15" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="31">
+        <v>41673</v>
+      </c>
+      <c r="D15" s="30">
+        <v>3.1440000000000001</v>
+      </c>
+      <c r="E15" s="32">
+        <v>304.8664</v>
+      </c>
+      <c r="F15" s="32">
+        <v>958.5</v>
+      </c>
+      <c r="G15" s="32"/>
+      <c r="H15" s="32"/>
+      <c r="J15" s="15">
+        <f>J14+D15</f>
+        <v>27.235999999999997</v>
+      </c>
+      <c r="K15" s="15"/>
+      <c r="L15" s="15"/>
+      <c r="M15" s="15"/>
+      <c r="O15" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A16" s="30">
+        <v>40</v>
+      </c>
+      <c r="B16" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="31">
+        <v>42047</v>
+      </c>
+      <c r="D16" s="30">
+        <v>15</v>
+      </c>
+      <c r="E16" s="32">
+        <v>457.97989999999999</v>
+      </c>
+      <c r="F16" s="32">
+        <v>6869.7</v>
+      </c>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="J16" s="15">
+        <f>J15-D16</f>
+        <v>12.235999999999997</v>
+      </c>
+      <c r="K16" s="15"/>
+      <c r="L16" s="15"/>
+      <c r="M16" s="15"/>
+      <c r="O16" s="46">
+        <f>(O9/D9*D16)</f>
+        <v>2.0859615793008062</v>
+      </c>
+      <c r="Q16" s="5">
+        <f>+O16*E14</f>
+        <v>522.41072107398907</v>
+      </c>
+      <c r="R16" s="5"/>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A17" s="30">
+        <v>96</v>
+      </c>
+      <c r="B17" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="31">
+        <v>42208</v>
+      </c>
+      <c r="D17" s="30">
+        <v>10.042999999999999</v>
+      </c>
+      <c r="E17" s="32">
+        <v>591.1232</v>
+      </c>
+      <c r="F17" s="32">
+        <v>5936.65</v>
+      </c>
+      <c r="G17" s="32"/>
+      <c r="H17" s="32"/>
+      <c r="J17" s="15">
+        <f>J16+D17</f>
+        <v>22.278999999999996</v>
+      </c>
+      <c r="L17" s="15"/>
+      <c r="R17" s="5"/>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A18" s="30">
+        <v>104</v>
+      </c>
+      <c r="B18" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="31">
+        <v>42311</v>
+      </c>
+      <c r="D18" s="30">
+        <v>4.7E-2</v>
+      </c>
+      <c r="E18" s="32">
+        <v>507.0213</v>
+      </c>
+      <c r="F18" s="32">
+        <v>23.83</v>
+      </c>
+      <c r="G18" s="32"/>
+      <c r="H18" s="32"/>
+      <c r="J18" s="15">
+        <f>J17+D18</f>
+        <v>22.325999999999997</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A19" s="30">
+        <v>202</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="31">
+        <v>44491</v>
+      </c>
+      <c r="D19" s="30">
+        <v>22.326000000000001</v>
+      </c>
+      <c r="E19" s="32">
+        <v>676.48</v>
+      </c>
+      <c r="F19" s="32">
+        <v>15103.09</v>
+      </c>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="J19" s="15">
+        <f>J18-D19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A20" s="47"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="45"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
+      <c r="J20" s="15"/>
+      <c r="N20" s="15"/>
+      <c r="O20" s="15"/>
+      <c r="P20" s="15"/>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A21" s="47"/>
+      <c r="B21" s="30"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="45"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="J21" s="15"/>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A22" s="47"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="45"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="32"/>
+      <c r="J22" s="15"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="J9 J16" formula="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AFDB5A1-07D9-4C61-B32E-B06B1CC9D3D5}">
   <dimension ref="A1:Q29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -813,7 +1503,7 @@
         <v>10</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H1" s="2"/>
       <c r="I1" s="2" t="s">
@@ -822,7 +1512,7 @@
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.35">
@@ -986,7 +1676,7 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D8" s="34"/>
       <c r="M8" s="5"/>
@@ -1033,7 +1723,7 @@
         <v>88</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C10" s="4">
         <v>42117</v>
@@ -1093,7 +1783,7 @@
         <v>0</v>
       </c>
       <c r="N11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.35">
@@ -1146,18 +1836,18 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D14" s="34"/>
       <c r="M14" s="5"/>
       <c r="O14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q14" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="P14" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="Q14" s="2" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.35">
@@ -1266,7 +1956,7 @@
         <v>87</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C17" s="4">
         <v>42136</v>
@@ -1583,7 +2273,7 @@
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.35">
       <c r="K26" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M26" s="29">
         <f>M7+M13+M24</f>
@@ -1611,9 +2301,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D44DFC7A-A8B1-46AB-BBD2-1EFF59E4C2EB}">
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1629,7 +2319,7 @@
     <col min="16" max="17" width="11.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="D1" t="s">
         <v>2</v>
       </c>
@@ -1643,9 +2333,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D2">
         <v>100</v>
@@ -1658,10 +2348,16 @@
         <v>1100</v>
       </c>
       <c r="G2" s="40"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="M2" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D3">
         <v>80</v>
@@ -1677,10 +2373,17 @@
         <f>D3*E3</f>
         <v>720</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L3" s="34"/>
+      <c r="M3" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D4">
         <v>20</v>
@@ -1696,20 +2399,32 @@
         <f>D4*E4</f>
         <v>260</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L4" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="M4" s="50">
+        <v>4195.84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="E5" s="40"/>
       <c r="F5" s="40"/>
       <c r="I5" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="J5" t="s">
         <v>44</v>
       </c>
-      <c r="J5" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L5" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="M5" s="50">
+        <v>70770.73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E6" s="40">
         <f>D3*E3-D3*E2</f>
@@ -1723,10 +2438,16 @@
       <c r="I6" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L6" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="M6" s="50">
+        <v>15658.2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E7" s="40">
         <f>D4*E4-D4*E2</f>
@@ -1740,10 +2461,18 @@
       <c r="I7" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L7" s="5"/>
+      <c r="M7" s="51">
+        <f>SUM(M4:M6)</f>
+        <v>90624.76999999999</v>
+      </c>
+      <c r="N7" s="51">
+        <v>89597.064809523305</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E8" s="40">
         <f>E6+D4*E4-D4*E2</f>
@@ -1755,62 +2484,69 @@
       </c>
       <c r="G8" s="40"/>
       <c r="I8" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+        <v>45</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N8" s="51">
+        <f>+M7-N7</f>
+        <v>1027.7051904766849</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C13">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C14">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>3</v>
       </c>
       <c r="B15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C15">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C16">
         <v>5</v>
       </c>
       <c r="E16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C17">
         <v>20</v>
       </c>
       <c r="E17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1819,13 +2555,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35931D83-0E0A-4D88-B489-4583A6E933E1}">
-  <dimension ref="A1:Q41"/>
+  <dimension ref="A1:R45"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.6328125" bestFit="1" customWidth="1"/>
@@ -1834,13 +2570,16 @@
     <col min="8" max="8" width="1.90625" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="7" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.54296875" customWidth="1"/>
-    <col min="15" max="15" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.54296875" customWidth="1"/>
+    <col min="16" max="16" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="11.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2" t="s">
@@ -1856,14 +2595,17 @@
         <v>10</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H1" s="2"/>
       <c r="I1" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="M1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" s="30">
         <v>79</v>
       </c>
@@ -1899,8 +2641,12 @@
         <f>+G3-G2</f>
         <v>167.73999999999978</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="M2" s="5">
+        <f>G3-G2</f>
+        <v>167.73999999999978</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="30">
         <v>80</v>
       </c>
@@ -1932,8 +2678,9 @@
         <f>J2-D3</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="M3" s="5"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" s="30">
         <v>81</v>
       </c>
@@ -1965,8 +2712,12 @@
         <f>J3+D4</f>
         <v>929</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="M4" s="5">
+        <f>G5-G4</f>
+        <v>192.80999999999949</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" s="30">
         <v>82</v>
       </c>
@@ -1998,8 +2749,9 @@
         <f>J4-D5</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="M5" s="5"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" s="30">
         <v>83</v>
       </c>
@@ -2031,8 +2783,12 @@
         <f t="shared" ref="J6:J25" si="0">J5+D6</f>
         <v>5386</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="M6" s="5">
+        <f>G7-G6</f>
+        <v>-1239.8400000000038</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="30">
         <v>84</v>
       </c>
@@ -2064,8 +2820,9 @@
         <f>J6-D7</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="M7" s="5"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" s="30">
         <v>94</v>
       </c>
@@ -2097,8 +2854,12 @@
         <f t="shared" si="0"/>
         <v>6415</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="M8" s="5">
+        <f>G9-G8</f>
+        <v>2499.7899999999936</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" s="30">
         <v>97</v>
       </c>
@@ -2130,13 +2891,14 @@
         <f>J8-D9</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="M9" s="5"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" s="30">
         <v>138</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>31</v>
+        <v>74</v>
       </c>
       <c r="C10" s="31">
         <v>42822</v>
@@ -2164,8 +2926,9 @@
         <v>0</v>
       </c>
       <c r="K10" s="5"/>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="M10" s="5"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" s="30">
         <v>151</v>
       </c>
@@ -2197,8 +2960,12 @@
         <f t="shared" si="0"/>
         <v>527</v>
       </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="M11" s="5">
+        <f>G12-G11</f>
+        <v>3985.2799999999988</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12" s="30">
         <v>165</v>
       </c>
@@ -2230,23 +2997,24 @@
         <f>J11-D12</f>
         <v>0</v>
       </c>
-      <c r="M12" s="2" t="s">
+      <c r="M12" s="5"/>
+      <c r="N12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O12" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="P12" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="O12" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="P12" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="R12" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13" s="30">
         <v>166</v>
       </c>
@@ -2286,27 +3054,31 @@
         <v>0</v>
       </c>
       <c r="M13" s="5">
+        <f>R13</f>
+        <v>-12190.883321275795</v>
+      </c>
+      <c r="N13" s="5">
         <f>F14+K13*E17</f>
         <v>26706.527999999998</v>
       </c>
-      <c r="N13" s="5">
+      <c r="O13" s="5">
         <f>I13+I14+I17/D17*K13</f>
         <v>46.219456869009583</v>
       </c>
-      <c r="O13" s="5">
+      <c r="P13" s="5">
         <f>E16/J16*K13</f>
         <v>169.60813559322034</v>
       </c>
-      <c r="P13" s="5">
-        <f>M13-F13</f>
+      <c r="Q13" s="5">
+        <f>N13-F13</f>
         <v>-12314.272000000004</v>
       </c>
-      <c r="Q13" s="5">
-        <f>P13-N13+O13</f>
+      <c r="R13" s="5">
+        <f>Q13-O13+P13</f>
         <v>-12190.883321275795</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" s="30">
         <v>169</v>
       </c>
@@ -2338,8 +3110,9 @@
         <f>J13-D14</f>
         <v>952</v>
       </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="M14" s="5"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15" s="30">
         <v>174</v>
       </c>
@@ -2375,13 +3148,14 @@
         <f>D15-(D17+D14-D13)</f>
         <v>400</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="M15" s="5"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A16" s="30">
         <v>176</v>
       </c>
       <c r="B16" s="30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C16" s="31">
         <v>43629</v>
@@ -2409,8 +3183,9 @@
         <v>1652</v>
       </c>
       <c r="M16" s="5"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N16" s="5"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A17" s="30">
         <v>177</v>
       </c>
@@ -2442,9 +3217,9 @@
         <f>J16-D17</f>
         <v>400</v>
       </c>
-      <c r="M17" s="34"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="M17" s="5"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A18" s="30">
         <v>178</v>
       </c>
@@ -2476,9 +3251,8 @@
         <f t="shared" si="0"/>
         <v>900</v>
       </c>
-      <c r="M18" s="34"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A19" s="30">
         <v>190</v>
       </c>
@@ -2511,8 +3285,9 @@
         <v>992</v>
       </c>
       <c r="K19" s="34"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="L19" s="34"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A20" s="30">
         <v>191</v>
       </c>
@@ -2549,7 +3324,7 @@
       </c>
       <c r="L20" s="34"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A21" s="30">
         <v>179</v>
       </c>
@@ -2584,7 +3359,7 @@
       <c r="K21" s="34"/>
       <c r="L21" s="34"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A22" s="30">
         <v>182</v>
       </c>
@@ -2623,8 +3398,9 @@
       <c r="L22" s="34">
         <v>67</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="M22" s="5"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A23" s="30">
         <v>192</v>
       </c>
@@ -2664,8 +3440,9 @@
         <f t="shared" ref="L23:L25" si="1">K23</f>
         <v>500</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="M23" s="5"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A24" s="30">
         <v>193</v>
       </c>
@@ -2705,13 +3482,14 @@
         <f t="shared" si="1"/>
         <v>433</v>
       </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="M24" s="5"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A25" s="30">
         <v>195</v>
       </c>
       <c r="B25" s="30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C25" s="31">
         <v>44362</v>
@@ -2746,8 +3524,9 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="M25" s="5"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A26" s="30">
         <v>206</v>
       </c>
@@ -2779,8 +3558,9 @@
         <f t="shared" ref="J26:J27" si="2">J25-D26</f>
         <v>1846</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="M26" s="5"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A27" s="30">
         <v>207</v>
       </c>
@@ -2812,8 +3592,9 @@
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="M27" s="5"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
       <c r="K28" s="41">
         <f>SUM(K20:K25)</f>
         <v>1900</v>
@@ -2823,342 +3604,442 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="E29" s="40"/>
-      <c r="F29" s="40"/>
-      <c r="G29" s="40"/>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="E30" s="40"/>
-      <c r="F30" s="40"/>
-      <c r="G30" s="40"/>
-      <c r="J30" s="1" t="s">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="K29" s="41"/>
+      <c r="L29" s="41" t="s">
+        <v>58</v>
+      </c>
+      <c r="M29" s="29">
+        <f>G2+G4+G6+G8+G11+G13+G15+G18+G19+G20+(D22-L22)*E22</f>
+        <v>209510.37</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="K30" s="41"/>
+      <c r="L30" s="41" t="s">
+        <v>57</v>
+      </c>
+      <c r="M30" s="29">
+        <f>G27+G26+G21+G17+G14+G12+G9+G7+G5+G3</f>
+        <v>215482.96999999997</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="E31" s="40"/>
+      <c r="F31" s="40"/>
+      <c r="G31" s="40"/>
+      <c r="L31" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="M31" s="29">
+        <f>+M30-M29</f>
+        <v>5972.5999999999767</v>
+      </c>
+      <c r="N31" s="5">
+        <v>5963.64</v>
+      </c>
+      <c r="O31" s="5">
+        <f>+M31-N31</f>
+        <v>8.9599999999763895</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="E32" s="40"/>
+      <c r="F32" s="40"/>
+      <c r="G32" s="40"/>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="E33" s="40"/>
+      <c r="F33" s="40"/>
+      <c r="G33" s="40"/>
+      <c r="J33" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="K30" s="1" t="s">
+      <c r="K33" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L30" s="1" t="s">
+      <c r="L33" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A31" s="30">
+      <c r="M33" s="1"/>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A34" s="30">
         <v>166</v>
       </c>
-      <c r="B31" s="30" t="s">
+      <c r="B34" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="C31" s="31">
+      <c r="C34" s="31">
         <v>43389</v>
       </c>
-      <c r="D31" s="33">
+      <c r="D34" s="33">
         <v>1600</v>
       </c>
-      <c r="E31" s="32">
+      <c r="E34" s="32">
         <v>24.388000000000002</v>
       </c>
-      <c r="F31" s="32">
+      <c r="F34" s="32">
         <v>39020.800000000003</v>
       </c>
-      <c r="G31" s="32">
+      <c r="G34" s="32">
         <v>39049.31</v>
       </c>
-      <c r="H31" s="30">
+      <c r="H34" s="30">
         <v>1</v>
       </c>
-      <c r="I31" s="32">
+      <c r="I34" s="32">
         <v>28.51</v>
       </c>
-      <c r="J31" s="34"/>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A32" s="30">
+      <c r="J34" s="34"/>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A35" s="30">
         <v>169</v>
       </c>
-      <c r="B32" s="30" t="s">
+      <c r="B35" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="C32" s="31">
+      <c r="C35" s="31">
         <v>43458</v>
       </c>
-      <c r="D32" s="33">
+      <c r="D35" s="33">
         <v>648</v>
       </c>
-      <c r="E32" s="32">
+      <c r="E35" s="32">
         <v>18.260000000000002</v>
       </c>
-      <c r="F32" s="32">
+      <c r="F35" s="32">
         <v>11832.48</v>
       </c>
-      <c r="G32" s="32">
+      <c r="G35" s="32">
         <v>11822.42</v>
       </c>
-      <c r="H32" s="30">
+      <c r="H35" s="30">
         <v>1</v>
       </c>
-      <c r="I32" s="32">
+      <c r="I35" s="32">
         <v>10.06</v>
       </c>
-      <c r="J32" s="32">
-        <f>G$31/D$31*D32</f>
+      <c r="J35" s="32">
+        <f>G$34/D$34*D35</f>
         <v>15814.970549999998</v>
       </c>
-      <c r="L32" s="5">
-        <f>+G32-J32</f>
+      <c r="L35" s="5">
+        <f>+G35-J35</f>
         <v>-3992.5505499999981</v>
       </c>
-      <c r="M32" s="5">
+      <c r="M35" s="5"/>
+      <c r="N35" s="5">
         <v>-3992.5505499999899</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A33" s="30">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A36" s="30">
         <v>177</v>
       </c>
-      <c r="B33" s="30" t="s">
+      <c r="B36" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="C33" s="31">
+      <c r="C36" s="31">
         <v>43797</v>
       </c>
-      <c r="D33" s="33">
-        <f>+D31-D32</f>
+      <c r="D36" s="33">
+        <f>+D34-D35</f>
         <v>952</v>
       </c>
-      <c r="E33" s="32">
+      <c r="E36" s="32">
         <v>15.624000000000001</v>
       </c>
-      <c r="F33" s="32">
-        <f>D33*E33</f>
+      <c r="F36" s="32">
+        <f>D36*E36</f>
         <v>14874.048000000001</v>
       </c>
-      <c r="G33" s="32">
-        <f>F33-I33</f>
+      <c r="G36" s="32">
+        <f>F36-I36</f>
         <v>14866.39854313099</v>
       </c>
-      <c r="H33" s="30">
+      <c r="H36" s="30">
         <v>1</v>
       </c>
-      <c r="I33" s="32">
-        <f>10.06/D17*D33</f>
+      <c r="I36" s="32">
+        <f>10.06/D17*D36</f>
         <v>7.6494568690095841</v>
       </c>
-      <c r="J33" s="32">
-        <f>G$31/D$31*D33</f>
+      <c r="J36" s="32">
+        <f>G$34/D$34*D36</f>
         <v>23234.339449999999</v>
       </c>
-      <c r="L33" s="5">
-        <f>+G33-J33</f>
+      <c r="L36" s="5">
+        <f>+G36-J36</f>
         <v>-8367.9409068690093</v>
       </c>
-      <c r="M33" s="5">
+      <c r="M36" s="5"/>
+      <c r="N36" s="5">
         <v>-8367.9409068690093</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="G34" s="5"/>
-      <c r="L34" s="29">
-        <f>SUM(L32:L33)</f>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="G37" s="5"/>
+      <c r="L37" s="29">
+        <f>SUM(L35:L36)</f>
         <v>-12360.491456869007</v>
       </c>
-      <c r="M34" s="29">
-        <f>SUM(M32:M33)</f>
+      <c r="M37" s="29"/>
+      <c r="N37" s="29">
+        <f>SUM(N35:N36)</f>
         <v>-12360.491456869</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="L36" t="s">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="L39" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="O36" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A37" s="30">
+      <c r="P39" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q39" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A40" s="30">
         <v>191</v>
       </c>
-      <c r="B37" s="30" t="s">
+      <c r="B40" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="C37" s="31">
+      <c r="C40" s="31">
         <v>43802</v>
       </c>
-      <c r="D37" s="33">
+      <c r="D40" s="33">
         <v>660</v>
       </c>
-      <c r="E37" s="32">
+      <c r="E40" s="32">
         <v>15.31</v>
       </c>
-      <c r="F37" s="32">
+      <c r="F40" s="32">
         <v>10104.6</v>
       </c>
-      <c r="G37" s="32">
+      <c r="G40" s="32">
         <v>10114.77</v>
-      </c>
-      <c r="H37" s="30">
-        <v>1</v>
-      </c>
-      <c r="I37" s="32">
-        <v>10.17</v>
-      </c>
-      <c r="J37" s="34">
-        <f>D37</f>
-        <v>660</v>
-      </c>
-      <c r="K37" s="34">
-        <v>400</v>
-      </c>
-      <c r="L37" s="5">
-        <f>-K37*E37-K37/D37*I37</f>
-        <v>-6130.1636363636362</v>
-      </c>
-      <c r="M37" s="43">
-        <f>G39</f>
-        <v>1543.79</v>
-      </c>
-      <c r="N37" s="46">
-        <f>(K37-D39)*E40</f>
-        <v>9895.6</v>
-      </c>
-      <c r="O37" s="29">
-        <f>SUM(L37:N37)</f>
-        <v>5309.2263636363641</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A38" s="30">
-        <v>182</v>
-      </c>
-      <c r="B38" s="30" t="s">
-        <v>5</v>
-      </c>
-      <c r="C38" s="31">
-        <v>43893</v>
-      </c>
-      <c r="D38" s="33">
-        <v>567</v>
-      </c>
-      <c r="E38" s="32">
-        <v>13.28</v>
-      </c>
-      <c r="F38" s="32">
-        <v>7529.76</v>
-      </c>
-      <c r="G38" s="32">
-        <v>7539.93</v>
-      </c>
-      <c r="H38" s="30">
-        <v>1</v>
-      </c>
-      <c r="I38" s="32">
-        <v>10.17</v>
-      </c>
-      <c r="J38" s="34">
-        <f>J37+D38</f>
-        <v>1227</v>
-      </c>
-      <c r="K38" s="34">
-        <f>D39+D40-K37</f>
-        <v>500</v>
-      </c>
-      <c r="L38" s="5">
-        <f>-K38*E38-K38/D38*I38</f>
-        <v>-6648.9682539682535</v>
-      </c>
-      <c r="N38" s="46">
-        <f>K38*E40</f>
-        <v>14300</v>
-      </c>
-      <c r="O38" s="29">
-        <f>SUM(L38:N38)</f>
-        <v>7651.0317460317465</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A39" s="44">
-        <v>206</v>
-      </c>
-      <c r="B39" s="30" t="s">
-        <v>6</v>
-      </c>
-      <c r="C39" s="31">
-        <v>44559</v>
-      </c>
-      <c r="D39" s="30">
-        <v>54</v>
-      </c>
-      <c r="E39" s="32">
-        <v>28.6</v>
-      </c>
-      <c r="F39" s="32">
-        <v>1544.4</v>
-      </c>
-      <c r="G39" s="32">
-        <v>1543.79</v>
-      </c>
-      <c r="H39" s="30">
-        <v>1</v>
-      </c>
-      <c r="I39" s="32">
-        <v>0.61</v>
-      </c>
-      <c r="J39" s="34">
-        <f>J38-D39</f>
-        <v>1173</v>
-      </c>
-      <c r="L39" s="5">
-        <f>G39</f>
-        <v>1543.79</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A40" s="45">
-        <v>207</v>
-      </c>
-      <c r="B40" s="30" t="s">
-        <v>6</v>
-      </c>
-      <c r="C40" s="31">
-        <v>44559</v>
-      </c>
-      <c r="D40" s="30">
-        <v>846</v>
-      </c>
-      <c r="E40" s="32">
-        <v>28.6</v>
-      </c>
-      <c r="F40" s="32">
-        <v>24195.599999999999</v>
-      </c>
-      <c r="G40" s="32">
-        <v>24186.04</v>
       </c>
       <c r="H40" s="30">
         <v>1</v>
       </c>
       <c r="I40" s="32">
+        <v>10.17</v>
+      </c>
+      <c r="J40" s="34">
+        <f>D40</f>
+        <v>660</v>
+      </c>
+      <c r="K40" s="34">
+        <v>400</v>
+      </c>
+      <c r="L40" s="5">
+        <f>-K40*E40</f>
+        <v>-6124</v>
+      </c>
+      <c r="M40" s="53">
+        <f>J40-K40</f>
+        <v>260</v>
+      </c>
+      <c r="N40" s="54">
+        <f>D43</f>
+        <v>54</v>
+      </c>
+      <c r="O40" s="55">
+        <f>D40-M40-N40</f>
+        <v>346</v>
+      </c>
+      <c r="P40" s="29">
+        <f>M40*E41+N40*E43+O40*E44-F40</f>
+        <v>5654.52</v>
+      </c>
+      <c r="Q40" s="29">
+        <v>5636.4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A41" s="52">
+        <v>179</v>
+      </c>
+      <c r="B41" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41" s="31">
+        <v>43872</v>
+      </c>
+      <c r="D41" s="33">
+        <v>1252</v>
+      </c>
+      <c r="E41" s="32">
+        <v>16.611999999999998</v>
+      </c>
+      <c r="F41" s="32">
+        <v>20798.22</v>
+      </c>
+      <c r="G41" s="32">
+        <v>20781.68</v>
+      </c>
+      <c r="H41" s="30">
+        <v>1</v>
+      </c>
+      <c r="I41" s="32">
+        <v>16.54</v>
+      </c>
+      <c r="J41" s="34">
+        <f>J40-D41</f>
+        <v>-592</v>
+      </c>
+      <c r="K41" s="34"/>
+      <c r="L41" s="34"/>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A42" s="30">
+        <v>182</v>
+      </c>
+      <c r="B42" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="C42" s="31">
+        <v>43893</v>
+      </c>
+      <c r="D42" s="33">
+        <v>567</v>
+      </c>
+      <c r="E42" s="32">
+        <v>13.28</v>
+      </c>
+      <c r="F42" s="32">
+        <v>7529.76</v>
+      </c>
+      <c r="G42" s="32">
+        <v>7539.93</v>
+      </c>
+      <c r="H42" s="30">
+        <v>1</v>
+      </c>
+      <c r="I42" s="32">
+        <v>10.17</v>
+      </c>
+      <c r="J42" s="34">
+        <f>J40+D42</f>
+        <v>1227</v>
+      </c>
+      <c r="K42" s="34">
+        <f>D43+D44-K40</f>
+        <v>500</v>
+      </c>
+      <c r="L42" s="5">
+        <f>-K42*E42</f>
+        <v>-6640</v>
+      </c>
+      <c r="M42" s="5"/>
+      <c r="O42" s="55">
+        <f>D44-O40</f>
+        <v>500</v>
+      </c>
+      <c r="P42" s="29">
+        <f>O42*E44+L42</f>
+        <v>7660</v>
+      </c>
+      <c r="Q42" s="29">
+        <v>7645.38</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A43" s="43">
+        <v>206</v>
+      </c>
+      <c r="B43" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="C43" s="31">
+        <v>44559</v>
+      </c>
+      <c r="D43" s="30">
+        <v>54</v>
+      </c>
+      <c r="E43" s="32">
+        <v>28.6</v>
+      </c>
+      <c r="F43" s="32">
+        <v>1544.4</v>
+      </c>
+      <c r="G43" s="32">
+        <v>1543.79</v>
+      </c>
+      <c r="H43" s="30">
+        <v>1</v>
+      </c>
+      <c r="I43" s="32">
+        <v>0.61</v>
+      </c>
+      <c r="J43" s="34">
+        <f>J42-D43</f>
+        <v>1173</v>
+      </c>
+      <c r="L43" s="5">
+        <f>G43</f>
+        <v>1543.79</v>
+      </c>
+      <c r="M43" s="5"/>
+      <c r="P43" s="5">
+        <f>SUM(P40:P42)</f>
+        <v>13314.52</v>
+      </c>
+      <c r="Q43" s="5">
+        <f>SUM(Q40:Q42)</f>
+        <v>13281.779999999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A44" s="44">
+        <v>207</v>
+      </c>
+      <c r="B44" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="C44" s="31">
+        <v>44559</v>
+      </c>
+      <c r="D44" s="30">
+        <v>846</v>
+      </c>
+      <c r="E44" s="32">
+        <v>28.6</v>
+      </c>
+      <c r="F44" s="32">
+        <v>24195.599999999999</v>
+      </c>
+      <c r="G44" s="32">
+        <v>24186.04</v>
+      </c>
+      <c r="H44" s="30">
+        <v>1</v>
+      </c>
+      <c r="I44" s="32">
         <v>9.56</v>
       </c>
-      <c r="J40" s="34">
-        <f>J39-D40</f>
+      <c r="J44" s="34">
+        <f>J43-D44</f>
         <v>327</v>
       </c>
-      <c r="L40" s="5">
-        <f>G40</f>
+      <c r="L44" s="5">
+        <f>G44</f>
         <v>24186.04</v>
       </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="L41" s="29">
-        <f>SUM(L37:L40)</f>
-        <v>12950.698109668112</v>
-      </c>
-      <c r="O41" s="29">
-        <f>SUM(O37:O40)</f>
-        <v>12960.25810966811</v>
-      </c>
+      <c r="M44" s="5"/>
+      <c r="Q44" s="5">
+        <f>+P43-Q43</f>
+        <v>32.740000000001601</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="I45" s="5"/>
+      <c r="P45" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3166,7 +4047,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2765C9F5-04DD-4DF6-B6C4-239116C295E5}">
   <dimension ref="A1:I100"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3449,7 +4330,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8A68C22-9B46-4722-8C3E-CFEEA15AC7BA}">
   <dimension ref="A1:J42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4232,7 +5113,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2C274DA-F909-48E4-B094-8A2D400FEEEF}">
   <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4434,7 +5315,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B93F3808-9942-41FF-8964-468989940CAA}">
   <dimension ref="B1:J28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Eliminada llista de PiG en cartera per anys i només poso el PiG actual.
</commit_message>
<xml_diff>
--- a/Docs/Proves-PiG Origen.xlsx
+++ b/Docs/Proves-PiG Origen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\Meus\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF39A4F-8DD9-4A1A-B8C2-E5C22E9D0CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F94242AC-9503-4EF3-8C6E-058F5DA2F0A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{A356EC3C-A36B-4D01-97F4-538073D64CD4}"/>
   </bookViews>
@@ -3648,7 +3648,7 @@
       <c r="F32" s="40"/>
       <c r="G32" s="40"/>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.35">
       <c r="E33" s="40"/>
       <c r="F33" s="40"/>
       <c r="G33" s="40"/>
@@ -3663,7 +3663,7 @@
       </c>
       <c r="M33" s="1"/>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A34" s="30">
         <v>166</v>
       </c>
@@ -3693,7 +3693,7 @@
       </c>
       <c r="J34" s="34"/>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A35" s="30">
         <v>169</v>
       </c>
@@ -3734,7 +3734,7 @@
         <v>-3992.5505499999899</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A36" s="30">
         <v>177</v>
       </c>
@@ -3779,7 +3779,7 @@
         <v>-8367.9409068690093</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.35">
       <c r="G37" s="5"/>
       <c r="L37" s="29">
         <f>SUM(L35:L36)</f>
@@ -3791,7 +3791,7 @@
         <v>-12360.491456869</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.35">
       <c r="L39" s="1" t="s">
         <v>7</v>
       </c>
@@ -3802,7 +3802,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A40" s="30">
         <v>191</v>
       </c>
@@ -3861,7 +3861,7 @@
         <v>5636.4</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A41" s="52">
         <v>179</v>
       </c>
@@ -3896,7 +3896,7 @@
       <c r="K41" s="34"/>
       <c r="L41" s="34"/>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A42" s="30">
         <v>182</v>
       </c>
@@ -3949,7 +3949,7 @@
         <v>7645.38</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A43" s="43">
         <v>206</v>
       </c>
@@ -3994,8 +3994,11 @@
         <f>SUM(Q40:Q42)</f>
         <v>13281.779999999999</v>
       </c>
-    </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="R43" s="32">
+        <v>467.17</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A44" s="44">
         <v>207</v>
       </c>
@@ -4037,7 +4040,7 @@
         <v>32.740000000001601</v>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.35">
       <c r="I45" s="5"/>
       <c r="P45" s="6"/>
     </row>

</xml_diff>

<commit_message>
En perdues i guanys tab poso totals a ntbPigCompra i ntbPigCompraOrig al seleccionar el producte.
</commit_message>
<xml_diff>
--- a/Docs/Proves-PiG Origen.xlsx
+++ b/Docs/Proves-PiG Origen.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\Meus\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F94242AC-9503-4EF3-8C6E-058F5DA2F0A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E7F2C63-C9F2-4E61-9155-066DF6CAB22C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{A356EC3C-A36B-4D01-97F4-538073D64CD4}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{A356EC3C-A36B-4D01-97F4-538073D64CD4}"/>
   </bookViews>
   <sheets>
     <sheet name="Asian Smaller" sheetId="10" r:id="rId1"/>

</xml_diff>

<commit_message>
-Afegit mètode desglosDeParticions utilitzat per compresDeParticions2 -Mètode desglosDeParticions el desgloç de les compres ara l'ordeno per data moviment i data moviment orig. -No permet modificat _ParticipacionsUtilitzades ni _ParticipacionsOcupades des del Moviment quan és una compra, s'ha de fer des del desgloç compra.
</commit_message>
<xml_diff>
--- a/Docs/Proves-PiG Origen.xlsx
+++ b/Docs/Proves-PiG Origen.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\Meus\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A24496E9-B130-480E-8C97-264B92C33BBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{409EFF10-19BA-4A35-8DF8-CABEDB7D4B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{A356EC3C-A36B-4D01-97F4-538073D64CD4}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="1" activeTab="4" xr2:uid="{A356EC3C-A36B-4D01-97F4-538073D64CD4}"/>
   </bookViews>
   <sheets>
     <sheet name="Biotechnology" sheetId="11" r:id="rId1"/>
@@ -984,7 +984,7 @@
       </c>
       <c r="G4" s="32"/>
       <c r="H4" s="15">
-        <f>H3+D4</f>
+        <f>IF(ISNUMBER(SEARCH("v",B4,1)),H3-D4,H3+D4)</f>
         <v>27.235999999999997</v>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="G5" s="32"/>
       <c r="H5" s="15">
-        <f>H4-D5</f>
+        <f>IF(ISNUMBER(SEARCH("v",B5,1)),H4-D5,H4+D5)</f>
         <v>12.235999999999997</v>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
         <v>5936.65</v>
       </c>
       <c r="H9" s="15">
-        <f>H8-D9</f>
+        <f t="shared" ref="H9:H10" si="0">IF(ISNUMBER(SEARCH("v",B9,1)),H8-D9,H8+D9)</f>
         <v>24.229000000000013</v>
       </c>
       <c r="I9">
@@ -1108,8 +1108,8 @@
         <v>1030.1199999999999</v>
       </c>
       <c r="H10" s="15">
-        <f>H9-D10</f>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1.4210854715202004E-14</v>
       </c>
       <c r="I10">
         <f>D10/D8*I8</f>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="G14" s="32"/>
       <c r="H14" s="15">
-        <f>H13+D14</f>
+        <f t="shared" ref="H14:H15" si="1">IF(ISNUMBER(SEARCH("v",B14,1)),H13-D14,H13+D14)</f>
         <v>22.325999999999997</v>
       </c>
     </row>
@@ -1212,8 +1212,8 @@
       </c>
       <c r="G15" s="32"/>
       <c r="H15" s="15">
-        <f>H14-D15</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>-3.5527136788005009E-15</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
@@ -1265,7 +1265,7 @@
         <v>15103.09</v>
       </c>
       <c r="H19" s="15">
-        <f t="shared" ref="H19:H20" si="0">H18+D19</f>
+        <f t="shared" ref="H19:H20" si="2">IF(ISNUMBER(SEARCH("v",B19,1)),H18-D19,H18+D19)</f>
         <v>59.263999999999996</v>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
         <v>20114.5</v>
       </c>
       <c r="H20" s="15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>105.53</v>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       <c r="G4" s="32"/>
       <c r="H4" s="32"/>
       <c r="J4" s="15">
-        <f>J3+D4</f>
+        <f>IF(ISNUMBER(SEARCH("v",B4,1)),J3-D4,J3+D4)</f>
         <v>1593.21</v>
       </c>
       <c r="K4" s="15">
@@ -1476,7 +1476,7 @@
       <c r="G5" s="32"/>
       <c r="H5" s="32"/>
       <c r="J5" s="15">
-        <f>J4+D5</f>
+        <f t="shared" ref="J5:J11" si="0">IF(ISNUMBER(SEARCH("v",B5,1)),J4-D5,J4+D5)</f>
         <v>2115.5839999999998</v>
       </c>
       <c r="K5" s="15"/>
@@ -1515,7 +1515,7 @@
       <c r="G6" s="32"/>
       <c r="H6" s="32"/>
       <c r="J6" s="15">
-        <f>J5-D6</f>
+        <f t="shared" si="0"/>
         <v>700.00199999999973</v>
       </c>
       <c r="L6" s="15"/>
@@ -1542,7 +1542,7 @@
       <c r="G7" s="32"/>
       <c r="H7" s="32"/>
       <c r="J7" s="15">
-        <f>J6-D7</f>
+        <f t="shared" si="0"/>
         <v>522.00199999999973</v>
       </c>
     </row>
@@ -1568,8 +1568,8 @@
       <c r="G8" s="32"/>
       <c r="H8" s="32"/>
       <c r="J8" s="15">
-        <f>J7-D8</f>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>-2.2737367544323206E-13</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.35">
@@ -1600,8 +1600,8 @@
         <v>457.97989999999999</v>
       </c>
       <c r="J9" s="15">
-        <f>J8+D9</f>
-        <v>174.22900000000001</v>
+        <f t="shared" si="0"/>
+        <v>174.22899999999979</v>
       </c>
       <c r="N9" s="15">
         <f>D10</f>
@@ -1643,8 +1643,8 @@
       <c r="G10" s="32"/>
       <c r="H10" s="32"/>
       <c r="J10" s="15">
-        <f>J9-D10</f>
-        <v>24.229000000000013</v>
+        <f t="shared" si="0"/>
+        <v>24.228999999999786</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.35">
@@ -1669,8 +1669,8 @@
       <c r="G11" s="32"/>
       <c r="H11" s="32"/>
       <c r="J11" s="15">
-        <f>J10-D11</f>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>-2.1316282072803006E-13</v>
       </c>
       <c r="R11" s="46"/>
     </row>
@@ -1732,7 +1732,7 @@
       <c r="G15" s="32"/>
       <c r="H15" s="32"/>
       <c r="J15" s="15">
-        <f>J14+D15</f>
+        <f t="shared" ref="J15:J19" si="1">IF(ISNUMBER(SEARCH("v",B15,1)),J14-D15,J14+D15)</f>
         <v>27.235999999999997</v>
       </c>
       <c r="K15" s="15"/>
@@ -1767,7 +1767,7 @@
       <c r="G16" s="32"/>
       <c r="H16" s="32"/>
       <c r="J16" s="15">
-        <f>J15-D16</f>
+        <f t="shared" si="1"/>
         <v>12.235999999999997</v>
       </c>
       <c r="K16" s="15"/>
@@ -1805,7 +1805,7 @@
       <c r="G17" s="32"/>
       <c r="H17" s="32"/>
       <c r="J17" s="15">
-        <f>J16+D17</f>
+        <f t="shared" si="1"/>
         <v>22.278999999999996</v>
       </c>
       <c r="L17" s="15"/>
@@ -1833,7 +1833,7 @@
       <c r="G18" s="32"/>
       <c r="H18" s="32"/>
       <c r="J18" s="15">
-        <f>J17+D18</f>
+        <f t="shared" si="1"/>
         <v>22.325999999999997</v>
       </c>
     </row>
@@ -1859,8 +1859,8 @@
       <c r="G19" s="32"/>
       <c r="H19" s="32"/>
       <c r="J19" s="15">
-        <f>J18-D19</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>-3.5527136788005009E-15</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.35">
@@ -1901,9 +1901,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="J9 J16" formula="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -3114,7 +3111,7 @@
         <v>25.32</v>
       </c>
       <c r="J3" s="34">
-        <f>J2-D3</f>
+        <f>IF(ISNUMBER(SEARCH("v",B3,1)),J2-D3,J2+D3)</f>
         <v>0</v>
       </c>
       <c r="M3" s="5"/>
@@ -3148,7 +3145,7 @@
         <v>15.06</v>
       </c>
       <c r="J4" s="34">
-        <f>J3+D4</f>
+        <f>IF(ISNUMBER(SEARCH("v",B4,1)),J3-D4,J3+D4)</f>
         <v>929</v>
       </c>
       <c r="M4" s="5">
@@ -3185,7 +3182,7 @@
         <v>15.09</v>
       </c>
       <c r="J5" s="34">
-        <f>J4-D5</f>
+        <f t="shared" ref="J5:J27" si="0">IF(ISNUMBER(SEARCH("v",B5,1)),J4-D5,J4+D5)</f>
         <v>0</v>
       </c>
       <c r="M5" s="5"/>
@@ -3219,7 +3216,7 @@
         <v>20.14</v>
       </c>
       <c r="J6" s="34">
-        <f t="shared" ref="J6:J25" si="0">J5+D6</f>
+        <f t="shared" si="0"/>
         <v>5386</v>
       </c>
       <c r="M6" s="5">
@@ -3256,7 +3253,7 @@
         <v>20.03</v>
       </c>
       <c r="J7" s="34">
-        <f>J6-D7</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="M7" s="5"/>
@@ -3327,7 +3324,7 @@
         <v>20.399999999999999</v>
       </c>
       <c r="J9" s="34">
-        <f>J8-D9</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="M9" s="5"/>
@@ -3361,7 +3358,6 @@
         <v>0</v>
       </c>
       <c r="J10" s="34">
-        <f>J9</f>
         <v>0</v>
       </c>
       <c r="K10" s="5"/>
@@ -3433,7 +3429,7 @@
         <v>27.45</v>
       </c>
       <c r="J12" s="34">
-        <f>J11-D12</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="M12" s="5"/>
@@ -3546,7 +3542,7 @@
         <v>10.06</v>
       </c>
       <c r="J14" s="34">
-        <f>J13-D14</f>
+        <f t="shared" si="0"/>
         <v>952</v>
       </c>
       <c r="M14" s="5"/>
@@ -3653,7 +3649,7 @@
         <v>10.06</v>
       </c>
       <c r="J17" s="34">
-        <f>J16-D17</f>
+        <f t="shared" si="0"/>
         <v>400</v>
       </c>
       <c r="M17" s="5"/>
@@ -3792,7 +3788,7 @@
         <v>16.54</v>
       </c>
       <c r="J21" s="34">
-        <f>J20-D21</f>
+        <f t="shared" si="0"/>
         <v>400</v>
       </c>
       <c r="K21" s="34"/>
@@ -3994,7 +3990,7 @@
         <v>0.61</v>
       </c>
       <c r="J26" s="34">
-        <f t="shared" ref="J26:J27" si="2">J25-D26</f>
+        <f t="shared" si="0"/>
         <v>1846</v>
       </c>
       <c r="M26" s="5"/>
@@ -4028,7 +4024,7 @@
         <v>9.56</v>
       </c>
       <c r="J27" s="34">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>1000</v>
       </c>
       <c r="M27" s="5"/>

</xml_diff>